<commit_message>
Add vacancy KPI and change scoring to 0-10
</commit_message>
<xml_diff>
--- a/Blue_Ribbon_BSC_Import_Template.xlsx
+++ b/Blue_Ribbon_BSC_Import_Template.xlsx
@@ -502,7 +502,7 @@
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>4. Manual RAG is optional. If populated it overrides the automated scoring rule. Hours Usage and Budget Variance now use configurable Target Range scoring.</t>
+          <t>4. Manual RAG is optional. If populated it overrides the automated scoring rule. Hours Usage and Budget Variance now use configurable Target Range scoring. Vacancies % is a service-level People KPI and can be entered manually or imported.</t>
         </is>
       </c>
     </row>
@@ -824,7 +824,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -1237,25 +1237,21 @@
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>HOURS_USAGE</t>
+          <t>VACANCY_PCT</t>
         </is>
       </c>
       <c r="E12" s="5" t="n">
-        <v>101.8</v>
-      </c>
-      <c r="F12" s="5" t="inlineStr">
-        <is>
-          <t>Green</t>
-        </is>
-      </c>
+        <v>4.4</v>
+      </c>
+      <c r="F12" s="5" t="n"/>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>Manual example until scoring logic agreed</t>
+          <t>Example vacancy percentage</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>Operations</t>
+          <t>People</t>
         </is>
       </c>
     </row>
@@ -1277,11 +1273,11 @@
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>BUDGET_VARIANCE</t>
+          <t>HOURS_USAGE</t>
         </is>
       </c>
       <c r="E13" s="5" t="n">
-        <v>-2.1</v>
+        <v>101.8</v>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
@@ -1290,12 +1286,12 @@
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>Manual example until finance scoring logic agreed</t>
+          <t>Manual example until scoring logic agreed</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>Operations</t>
         </is>
       </c>
     </row>
@@ -1307,23 +1303,35 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Group</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr"/>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>WILLOW</t>
+        </is>
+      </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>OCCUPANCY</t>
+          <t>BUDGET_VARIANCE</t>
         </is>
       </c>
       <c r="E14" s="5" t="n">
-        <v>91.5</v>
-      </c>
-      <c r="F14" s="5" t="inlineStr"/>
-      <c r="G14" s="5" t="inlineStr"/>
+        <v>-2.1</v>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>Green</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>Manual example until finance scoring logic agreed</t>
+        </is>
+      </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>Operations</t>
+          <t>Finance</t>
         </is>
       </c>
     </row>
@@ -1335,31 +1343,23 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Service</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>WILLOW</t>
-        </is>
-      </c>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr"/>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>NPS_SCORE</t>
+          <t>OCCUPANCY</t>
         </is>
       </c>
       <c r="E15" s="5" t="n">
-        <v>42</v>
-      </c>
-      <c r="F15" s="5" t="n"/>
-      <c r="G15" s="5" t="inlineStr">
-        <is>
-          <t>Example NPS score</t>
-        </is>
-      </c>
+        <v>91.5</v>
+      </c>
+      <c r="F15" s="5" t="inlineStr"/>
+      <c r="G15" s="5" t="inlineStr"/>
       <c r="H15" s="5" t="inlineStr">
         <is>
-          <t>People</t>
+          <t>Operations</t>
         </is>
       </c>
     </row>
@@ -1371,25 +1371,61 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Group</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="n"/>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>WILLOW</t>
+        </is>
+      </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
           <t>NPS_SCORE</t>
         </is>
       </c>
       <c r="E16" s="5" t="n">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="F16" s="5" t="n"/>
       <c r="G16" s="5" t="inlineStr">
         <is>
+          <t>Example NPS score</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>People</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="n"/>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>NPS_SCORE</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="n">
+        <v>36</v>
+      </c>
+      <c r="F17" s="5" t="n"/>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
           <t>Example group NPS score</t>
         </is>
       </c>
-      <c r="H16" s="5" t="inlineStr">
+      <c r="H17" s="5" t="inlineStr">
         <is>
           <t>People</t>
         </is>
@@ -1415,7 +1451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -1884,17 +1920,17 @@
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>OCCUPANCY</t>
+          <t>VACANCY_PCT</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>Occupancy</t>
+          <t>Vacancies %</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>Operations</t>
+          <t>People</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
@@ -1904,35 +1940,35 @@
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>Higher is better</t>
+          <t>Lower is better</t>
         </is>
       </c>
       <c r="F12" s="7" t="n"/>
       <c r="G12" s="7" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H12" s="7" t="inlineStr">
         <is>
-          <t>85</t>
+          <t>10</t>
         </is>
       </c>
       <c r="I12" s="7" t="inlineStr">
         <is>
-          <t>Group only; example threshold only</t>
+          <t>Starter thresholds: Green &lt;= 5%; Amber &gt; 5% to 10%; Red &gt; 10%. Configurable in KPI Setup.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>HOURS_USAGE</t>
+          <t>OCCUPANCY</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>Hours Usage</t>
+          <t>Occupancy</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
@@ -1947,38 +1983,40 @@
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>Target Range</t>
-        </is>
-      </c>
-      <c r="F13" s="7" t="n">
-        <v>100</v>
-      </c>
-      <c r="G13" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="H13" s="7" t="n">
-        <v>5</v>
+          <t>Higher is better</t>
+        </is>
+      </c>
+      <c r="F13" s="7" t="n"/>
+      <c r="G13" s="7" t="inlineStr">
+        <is>
+          <t>90</t>
+        </is>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>85</t>
+        </is>
       </c>
       <c r="I13" s="7" t="inlineStr">
         <is>
-          <t>Target 100%. Green within +/-2%; Amber within +/-5%; Red outside +/-5%.</t>
+          <t>Group only; example threshold only</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>BUDGET_VARIANCE</t>
+          <t>HOURS_USAGE</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>Budget Over / Underspend</t>
+          <t>Hours Usage</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>Operations</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
@@ -1992,7 +2030,7 @@
         </is>
       </c>
       <c r="F14" s="7" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="G14" s="7" t="n">
         <v>2</v>
@@ -2002,48 +2040,89 @@
       </c>
       <c r="I14" s="7" t="inlineStr">
         <is>
-          <t>Target 0%. Green within +/-2%; Amber within +/-5%; Red outside +/-5%.</t>
+          <t>Target 100%. Green within +/-2%; Amber within +/-5%; Red outside +/-5%.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
+          <t>BUDGET_VARIANCE</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Budget Over / Underspend</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>Target Range</t>
+        </is>
+      </c>
+      <c r="F15" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="H15" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="I15" s="7" t="inlineStr">
+        <is>
+          <t>Target 0%. Green within +/-2%; Amber within +/-5%; Red outside +/-5%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
           <t>NPS_SCORE</t>
         </is>
       </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B16" s="7" t="inlineStr">
         <is>
           <t>NPS Score</t>
         </is>
       </c>
-      <c r="C15" s="7" t="inlineStr">
+      <c r="C16" s="7" t="inlineStr">
         <is>
           <t>People</t>
         </is>
       </c>
-      <c r="D15" s="7" t="inlineStr">
+      <c r="D16" s="7" t="inlineStr">
         <is>
           <t>Score</t>
         </is>
       </c>
-      <c r="E15" s="7" t="inlineStr">
+      <c r="E16" s="7" t="inlineStr">
         <is>
           <t>Higher is better</t>
         </is>
       </c>
-      <c r="F15" s="7" t="n"/>
-      <c r="G15" s="7" t="inlineStr">
+      <c r="F16" s="7" t="n"/>
+      <c r="G16" s="7" t="inlineStr">
         <is>
           <t>50</t>
         </is>
       </c>
-      <c r="H15" s="7" t="inlineStr">
+      <c r="H16" s="7" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="I15" s="7" t="inlineStr">
+      <c r="I16" s="7" t="inlineStr">
         <is>
           <t>Starter thresholds: Green &gt;= 50; Amber 0 to 49.9; Red &lt; 0. Configurable in KPI Setup.</t>
         </is>

</xml_diff>